<commit_message>
Updated ITA_grids_syn_5 model - 2025-10-20 15:28
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE74DCBF-1A57-46B7-A804-B37D3F254B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E39EB8CC-B717-4E58-969B-BFC96712948A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9265,7 +9265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A550F234-D447-4262-A97A-4C5810420BA7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D64E58C-688F-4D52-83B4-07BB68E05C65}">
   <dimension ref="B9:H144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11983,7 +11983,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35934413-0817-46FB-9FF4-25294C06B1C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE406493-4580-4953-AAE8-549F63618379}">
   <dimension ref="B9:L144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_syn_5 model - 2025-10-20 15:48
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E39EB8CC-B717-4E58-969B-BFC96712948A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5F55750-5234-4A90-BD18-EEDF6402873A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9265,7 +9265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D64E58C-688F-4D52-83B4-07BB68E05C65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348C70C5-9AB0-4936-B402-0991A4FC3999}">
   <dimension ref="B9:H144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11983,7 +11983,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE406493-4580-4953-AAE8-549F63618379}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C25185D-63FE-45E2-84F0-3373AB9C0077}">
   <dimension ref="B9:L144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_syn_5 model - 2025-11-05 18:54
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5F55750-5234-4A90-BD18-EEDF6402873A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5719F63-A6CB-48E4-8678-86CAEF94467C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9265,7 +9265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348C70C5-9AB0-4936-B402-0991A4FC3999}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40BEB547-C772-4883-BD4A-692F3BF32966}">
   <dimension ref="B9:H144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11983,7 +11983,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C25185D-63FE-45E2-84F0-3373AB9C0077}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB4A4EA-866C-42E8-86AB-7F289EAE8E51}">
   <dimension ref="B9:L144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_syn_5 model - 2025-11-19 15:39
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A85D7490-28EF-4779-995F-C4AD2A08C308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A323CB8-8EAC-4C92-84F3-784A7258D2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28277,7 +28277,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA6B8596-60DC-40E4-8D54-FFBDE07D0195}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C17642CE-8DF6-4F7A-91B0-9EBE58074D03}">
   <dimension ref="B9:H144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30995,7 +30995,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABD766B6-49F9-4CE9-9812-0972A076B471}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21E484A-4837-4033-A7EE-669952E1A252}">
   <dimension ref="B9:L144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_syn_5 model - 2025-11-19 16:02
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_syn_5/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A323CB8-8EAC-4C92-84F3-784A7258D2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{052BA3E4-D3B5-44DD-B4E3-6185755360AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28277,7 +28277,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C17642CE-8DF6-4F7A-91B0-9EBE58074D03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAC05FCF-EFFE-422C-B775-C428C837A4E0}">
   <dimension ref="B9:H144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30995,7 +30995,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21E484A-4837-4033-A7EE-669952E1A252}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{836A5067-F426-438A-8CE1-02689919B158}">
   <dimension ref="B9:L144"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>